<commit_message>
Feat/dodge action animation (#46)
* 구르기 액션 애니메이션과 스태미너 흐름을 정리

* 구르기 연속 재생 콜백과 입력 버퍼를 동기화

* 구르기: 입력 방향 기반 연속 재생 처리
</commit_message>
<xml_diff>
--- a/BADesign/Excel/Action.xlsx
+++ b/BADesign/Excel/Action.xlsx
@@ -975,6 +975,18 @@
           <t>DodgeRoll</t>
         </is>
       </c>
+      <c r="J7" s="0" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" s="0" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1145,7 +1157,7 @@
         <v>0.1</v>
       </c>
       <c r="L3" s="0" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1159,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.6640625" customWidth="1" style="2" min="1" max="1"/>
@@ -1247,12 +1259,50 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="0" t="n">
+        <v>40022</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>30021</v>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>InterruptLock</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="3" t="n"/>
+      <c r="F4" s="0" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="n">
+        <v>40023</v>
+      </c>
+      <c r="C5" t="n">
+        <v>30021</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>InputBuffer</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Features/skill dodge - fix (#61)
* 플레이어, 컴포넌트 주석 작성

* PlayerSkillComponent 생성

* 디스패처 함수 추가

* Look y축 방향 negate

* 주석 추가

* 뒤구르기 추가 및 테스트

* 스킬트리 여는 인풋 추가

* 스킬트리 창 닫힐 때 델리게이트 연결

- LayerBase::OnPopped 오버라이드하여 델리게이트 연결
- AnimMontage 경로 수정 및 추가
- IMC 추가: 임시 - 체크포인트에서만 활성화되도록 수정 필요

* 전진 대시

* Direction 카메라 방향 -> 플레이어 방향으로 수정

* AnimMontage 방향별로 연결

* OnDamaged 함수 준비(TODO)

* 버그 수정중
방향키 없이 입력 시 전진은 되는 상태
루트모션의 회전이 들어감

* 루트모션-애니메이션 윈도우 버그 수정

- 엑셀 데이터 수정
- 잘못 접근한 버그 수정 코드 롤백
- TODO1: 기본 카메라 모드에서 애니메이션 방향이 2배로 적용되는 버그 수정
- TODO2: 대시 윈도우 값 조정(ActionData 값과 불일치)

* 회피 방향 버그 수정

- Strafe 상태가 아닐 때 방향 기본값 Any로 지정

* 스킬 해제 추가, 엑셀 데이터 추가

---------

Co-authored-by: JinHyeok <kksd2950@gmail.com>
</commit_message>
<xml_diff>
--- a/BADesign/Excel/Action.xlsx
+++ b/BADesign/Excel/Action.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="79">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t xml:space="preserve">/Game/Character/Player/Animation/Montages/DodgeRoll/AM_Roll_Relaxed_Forward.AM_Roll_Relaxed_Forward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forward</t>
   </si>
   <si>
     <t xml:space="preserve">Backward</t>
@@ -277,19 +280,16 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="12"/>
@@ -609,37 +609,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285f4"/>
+        <a:srgbClr val="4285F4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ea4335"/>
+        <a:srgbClr val="EA4335"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="fbbc04"/>
+        <a:srgbClr val="FBBC04"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34a853"/>
+        <a:srgbClr val="34A853"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="ff6d01"/>
+        <a:srgbClr val="FF6D01"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46bdc6"/>
+        <a:srgbClr val="46BDC6"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Sheets">
@@ -779,7 +779,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N8"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.62109375" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.08"/>
@@ -1115,7 +1115,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="7.68359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="7.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="5.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="8.94"/>
@@ -1366,8 +1366,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultColWidth="7.69140625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr defaultColWidth="7.6875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="9.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="14.38"/>
@@ -1378,7 +1378,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="17" width="12.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="17" width="11.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="17" width="10.87"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="13" style="17" width="7.69"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="13" style="17" width="7.68"/>
   </cols>
   <sheetData>
     <row r="1" s="20" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1493,13 +1493,13 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="0" t="n">
         <v>30022</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="0" t="n">
         <v>10021</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="0" t="s">
         <v>48</v>
       </c>
       <c r="E4" s="26" t="s">
@@ -1508,16 +1508,17 @@
       <c r="F4" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="I4" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K4" s="17" t="n">
+      <c r="G4" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="0"/>
+      <c r="I4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>0.1</v>
       </c>
       <c r="L4" s="12" t="b">
@@ -1526,14 +1527,14 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="26" t="n">
+      <c r="B5" s="17" t="n">
         <v>30023</v>
       </c>
-      <c r="C5" s="26" t="n">
+      <c r="C5" s="17" t="n">
         <v>10021</v>
       </c>
-      <c r="D5" s="27" t="s">
-        <v>50</v>
+      <c r="D5" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>37</v>
@@ -1542,15 +1543,15 @@
         <v>39</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="I5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K5" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K5" s="17" t="n">
         <v>0.1</v>
       </c>
       <c r="L5" s="12" t="b">
@@ -1562,11 +1563,11 @@
       <c r="B6" s="17" t="n">
         <v>30024</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="26" t="n">
         <v>10021</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>37</v>
@@ -1575,15 +1576,15 @@
         <v>39</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K6" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>0.1</v>
       </c>
       <c r="L6" s="12" t="b">
@@ -1595,11 +1596,11 @@
       <c r="B7" s="26" t="n">
         <v>30025</v>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C7" s="17" t="n">
         <v>10021</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>37</v>
@@ -1608,15 +1609,15 @@
         <v>39</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K7" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K7" s="17" t="n">
         <v>0.1</v>
       </c>
       <c r="L7" s="12" t="b">
@@ -1628,11 +1629,11 @@
       <c r="B8" s="17" t="n">
         <v>30026</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="26" t="n">
         <v>10021</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>37</v>
@@ -1641,15 +1642,15 @@
         <v>39</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="I8" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K8" s="17" t="n">
+        <v>56</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K8" s="12" t="n">
         <v>0.1</v>
       </c>
       <c r="L8" s="12" t="b">
@@ -1661,11 +1662,11 @@
       <c r="B9" s="26" t="n">
         <v>30027</v>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="17" t="n">
         <v>10021</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>37</v>
@@ -1674,15 +1675,15 @@
         <v>39</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="I9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K9" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K9" s="17" t="n">
         <v>0.1</v>
       </c>
       <c r="L9" s="12" t="b">
@@ -1694,11 +1695,11 @@
       <c r="B10" s="26" t="n">
         <v>30028</v>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="26" t="n">
         <v>10021</v>
       </c>
       <c r="D10" s="27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>37</v>
@@ -1707,15 +1708,15 @@
         <v>39</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>61</v>
-      </c>
-      <c r="I10" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K10" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>0.1</v>
       </c>
       <c r="L10" s="12" t="b">
@@ -1724,19 +1725,19 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="0" t="n">
         <v>30029</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>10022</v>
+        <v>10021</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="27" t="s">
+      <c r="F11" s="12" t="s">
         <v>39</v>
       </c>
       <c r="G11" s="27" t="s">
@@ -1760,11 +1761,11 @@
       <c r="B12" s="26" t="n">
         <v>30030</v>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="0" t="n">
         <v>10022</v>
       </c>
-      <c r="D12" s="12" t="s">
-        <v>48</v>
+      <c r="D12" s="0" t="s">
+        <v>39</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>37</v>
@@ -1775,13 +1776,14 @@
       <c r="G12" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="I12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K12" s="12" t="n">
+      <c r="H12" s="0"/>
+      <c r="I12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K12" s="17" t="n">
         <v>0.1</v>
       </c>
       <c r="L12" s="12" t="b">
@@ -1797,16 +1799,16 @@
         <v>10022</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="27" t="s">
         <v>39</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I13" s="17" t="n">
         <v>1</v>
@@ -1829,8 +1831,8 @@
       <c r="C14" s="17" t="n">
         <v>10022</v>
       </c>
-      <c r="D14" s="27" t="s">
-        <v>52</v>
+      <c r="D14" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E14" s="26" t="s">
         <v>37</v>
@@ -1839,7 +1841,7 @@
         <v>39</v>
       </c>
       <c r="G14" s="27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I14" s="12" t="n">
         <v>1</v>
@@ -1863,7 +1865,7 @@
         <v>10022</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E15" s="26" t="s">
         <v>37</v>
@@ -1872,7 +1874,7 @@
         <v>39</v>
       </c>
       <c r="G15" s="27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I15" s="17" t="n">
         <v>1</v>
@@ -1896,7 +1898,7 @@
         <v>10022</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E16" s="26" t="s">
         <v>37</v>
@@ -1905,7 +1907,7 @@
         <v>39</v>
       </c>
       <c r="G16" s="27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I16" s="12" t="n">
         <v>1</v>
@@ -1929,7 +1931,7 @@
         <v>10022</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E17" s="26" t="s">
         <v>37</v>
@@ -1938,7 +1940,7 @@
         <v>39</v>
       </c>
       <c r="G17" s="27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I17" s="17" t="n">
         <v>1</v>
@@ -1962,7 +1964,7 @@
         <v>10022</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E18" s="26" t="s">
         <v>37</v>
@@ -1971,7 +1973,7 @@
         <v>39</v>
       </c>
       <c r="G18" s="27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I18" s="12" t="n">
         <v>1</v>
@@ -1988,9 +1990,70 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="12"/>
+      <c r="B19" s="0" t="n">
+        <v>30037</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>10022</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G19" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L19" s="12" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="0" t="n">
+        <v>30038</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>10022</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G20" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K20" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L20" s="12" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2008,7 +2071,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr defaultColWidth="7.703125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="7.51"/>
@@ -2051,19 +2114,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2075,7 +2138,7 @@
         <v>30021</v>
       </c>
       <c r="D3" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E3" s="33" t="n">
         <v>0.1</v>
@@ -2094,7 +2157,7 @@
         <v>30021</v>
       </c>
       <c r="D4" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E4" s="34" t="n">
         <v>0</v>
@@ -2113,7 +2176,7 @@
         <v>30021</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E5" s="36" t="n">
         <v>0.55</v>
@@ -2131,7 +2194,7 @@
         <v>30022</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>0.1</v>
@@ -2148,7 +2211,7 @@
         <v>30022</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>0</v>
@@ -2165,7 +2228,7 @@
         <v>30022</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E8" s="36" t="n">
         <v>0.55</v>
@@ -2182,7 +2245,7 @@
         <v>30023</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E9" s="33" t="n">
         <v>0.1</v>
@@ -2199,7 +2262,7 @@
         <v>30023</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>0</v>
@@ -2216,7 +2279,7 @@
         <v>30023</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>0.55</v>
@@ -2233,7 +2296,7 @@
         <v>30024</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E12" s="33" t="n">
         <v>0.1</v>
@@ -2250,7 +2313,7 @@
         <v>30024</v>
       </c>
       <c r="D13" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>0</v>
@@ -2267,7 +2330,7 @@
         <v>30024</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E14" s="36" t="n">
         <v>0.55</v>
@@ -2284,7 +2347,7 @@
         <v>30025</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E15" s="33" t="n">
         <v>0.1</v>
@@ -2301,7 +2364,7 @@
         <v>30025</v>
       </c>
       <c r="D16" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E16" s="34" t="n">
         <v>0</v>
@@ -2318,7 +2381,7 @@
         <v>30025</v>
       </c>
       <c r="D17" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E17" s="36" t="n">
         <v>0.55</v>
@@ -2335,7 +2398,7 @@
         <v>30026</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E18" s="33" t="n">
         <v>0.1</v>
@@ -2352,7 +2415,7 @@
         <v>30026</v>
       </c>
       <c r="D19" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E19" s="34" t="n">
         <v>0</v>
@@ -2369,7 +2432,7 @@
         <v>30026</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E20" s="36" t="n">
         <v>0.55</v>
@@ -2386,7 +2449,7 @@
         <v>30027</v>
       </c>
       <c r="D21" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E21" s="33" t="n">
         <v>0.1</v>
@@ -2403,7 +2466,7 @@
         <v>30027</v>
       </c>
       <c r="D22" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E22" s="34" t="n">
         <v>0</v>
@@ -2420,7 +2483,7 @@
         <v>30027</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E23" s="36" t="n">
         <v>0.55</v>
@@ -2437,7 +2500,7 @@
         <v>30028</v>
       </c>
       <c r="D24" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E24" s="33" t="n">
         <v>0.1</v>
@@ -2454,7 +2517,7 @@
         <v>30028</v>
       </c>
       <c r="D25" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E25" s="34" t="n">
         <v>0</v>
@@ -2471,7 +2534,7 @@
         <v>30028</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E26" s="36" t="n">
         <v>0.55</v>
@@ -2488,7 +2551,7 @@
         <v>30029</v>
       </c>
       <c r="D27" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E27" s="33" t="n">
         <v>0.1</v>
@@ -2505,7 +2568,7 @@
         <v>30029</v>
       </c>
       <c r="D28" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E28" s="34" t="n">
         <v>0</v>
@@ -2522,7 +2585,7 @@
         <v>30029</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E29" s="36" t="n">
         <v>0.55</v>
@@ -2539,7 +2602,7 @@
         <v>30030</v>
       </c>
       <c r="D30" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E30" s="33" t="n">
         <v>0.1</v>
@@ -2556,7 +2619,7 @@
         <v>30030</v>
       </c>
       <c r="D31" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E31" s="34" t="n">
         <v>0</v>
@@ -2573,7 +2636,7 @@
         <v>30030</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E32" s="36" t="n">
         <v>0.55</v>
@@ -2590,7 +2653,7 @@
         <v>30031</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E33" s="33" t="n">
         <v>0.1</v>
@@ -2607,7 +2670,7 @@
         <v>30031</v>
       </c>
       <c r="D34" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E34" s="34" t="n">
         <v>0</v>
@@ -2624,7 +2687,7 @@
         <v>30031</v>
       </c>
       <c r="D35" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E35" s="36" t="n">
         <v>0.55</v>
@@ -2641,7 +2704,7 @@
         <v>30032</v>
       </c>
       <c r="D36" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E36" s="33" t="n">
         <v>0.1</v>
@@ -2658,7 +2721,7 @@
         <v>30032</v>
       </c>
       <c r="D37" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E37" s="34" t="n">
         <v>0</v>
@@ -2675,7 +2738,7 @@
         <v>30032</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E38" s="36" t="n">
         <v>0.55</v>
@@ -2692,7 +2755,7 @@
         <v>30033</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E39" s="33" t="n">
         <v>0.1</v>
@@ -2709,7 +2772,7 @@
         <v>30033</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E40" s="34" t="n">
         <v>0</v>
@@ -2726,7 +2789,7 @@
         <v>30033</v>
       </c>
       <c r="D41" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E41" s="36" t="n">
         <v>0.55</v>
@@ -2743,7 +2806,7 @@
         <v>30034</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E42" s="33" t="n">
         <v>0.1</v>
@@ -2760,7 +2823,7 @@
         <v>30034</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E43" s="34" t="n">
         <v>0</v>
@@ -2777,7 +2840,7 @@
         <v>30034</v>
       </c>
       <c r="D44" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E44" s="36" t="n">
         <v>0.55</v>
@@ -2794,7 +2857,7 @@
         <v>30035</v>
       </c>
       <c r="D45" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E45" s="33" t="n">
         <v>0.1</v>
@@ -2811,7 +2874,7 @@
         <v>30035</v>
       </c>
       <c r="D46" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E46" s="34" t="n">
         <v>0</v>
@@ -2828,7 +2891,7 @@
         <v>30035</v>
       </c>
       <c r="D47" s="36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E47" s="36" t="n">
         <v>0.55</v>
@@ -2845,7 +2908,7 @@
         <v>30036</v>
       </c>
       <c r="D48" s="33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E48" s="33" t="n">
         <v>0.1</v>
@@ -2862,7 +2925,7 @@
         <v>30036</v>
       </c>
       <c r="D49" s="34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E49" s="34" t="n">
         <v>0</v>
@@ -2879,12 +2942,114 @@
         <v>30036</v>
       </c>
       <c r="D50" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="E50" s="36" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F50" s="36" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="17" t="n">
+        <v>40069</v>
+      </c>
+      <c r="C51" s="17" t="n">
+        <v>30037</v>
+      </c>
+      <c r="D51" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="E51" s="33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F51" s="34" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="17" t="n">
+        <v>40070</v>
+      </c>
+      <c r="C52" s="17" t="n">
+        <v>30037</v>
+      </c>
+      <c r="D52" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="E50" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F50" s="36" t="n">
+      <c r="E52" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="34" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="17" t="n">
+        <v>40071</v>
+      </c>
+      <c r="C53" s="17" t="n">
+        <v>30037</v>
+      </c>
+      <c r="D53" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="E53" s="36" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F53" s="36" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="36" t="n">
+        <v>40072</v>
+      </c>
+      <c r="C54" s="17" t="n">
+        <v>30038</v>
+      </c>
+      <c r="D54" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="E54" s="33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F54" s="34" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="17" t="n">
+        <v>40073</v>
+      </c>
+      <c r="C55" s="17" t="n">
+        <v>30038</v>
+      </c>
+      <c r="D55" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="E55" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="34" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="17" t="n">
+        <v>40074</v>
+      </c>
+      <c r="C56" s="17" t="n">
+        <v>30038</v>
+      </c>
+      <c r="D56" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="E56" s="36" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F56" s="36" t="n">
         <v>0.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
플레이어에 CombatComponent 추가, EnemyBase->CharacterBase 변경 중
</commit_message>
<xml_diff>
--- a/BADesign/Excel/Action.xlsx
+++ b/BADesign/Excel/Action.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ActionData" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="80">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t xml:space="preserve">/Game/Character/Player/Animation/Montages/DodgeRoll/AM_Dodge_Relaxed_BackwardRight.AM_Dodge_Relaxed_BackwardRight</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">ActionAnimationTid</t>
@@ -326,7 +329,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -342,7 +345,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFFFF5CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFD7"/>
+        <bgColor rgb="FFFFF5CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF5CE"/>
+        <bgColor rgb="FFFFFFD7"/>
       </patternFill>
     </fill>
   </fills>
@@ -380,7 +395,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -481,15 +496,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -558,7 +597,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFFFD7"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -575,7 +614,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFF5CE"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -1366,8 +1405,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultColWidth="7.6875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L22"/>
+  <sheetFormatPr defaultColWidth="7.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="9.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="14.38"/>
@@ -1457,7 +1496,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25"/>
       <c r="B3" s="25" t="n">
         <v>30021</v>
@@ -1471,588 +1510,591 @@
       <c r="E3" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="27" t="s">
         <v>39</v>
       </c>
       <c r="G3" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L3" s="12" t="b">
+      <c r="H3" s="27"/>
+      <c r="I3" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K3" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L3" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="n">
+    <row r="4" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="28" t="n">
         <v>30022</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="28" t="s">
         <v>48</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="27" t="s">
         <v>39</v>
       </c>
       <c r="G4" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="0"/>
-      <c r="I4" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L4" s="12" t="b">
+      <c r="I4" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K4" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L4" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="17" t="n">
+    <row r="5" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="28" t="n">
         <v>30023</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="27" t="s">
         <v>49</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G5" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K5" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L5" s="12" t="b">
+      <c r="I5" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K5" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L5" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="17" t="n">
+    <row r="6" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="28" t="n">
         <v>30024</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>10021</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="D6" s="29" t="s">
         <v>51</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="I6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L6" s="12" t="b">
+      <c r="I6" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K6" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L6" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="26" t="n">
         <v>30025</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" s="29" t="s">
         <v>53</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G7" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="I7" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K7" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L7" s="12" t="b">
+      <c r="I7" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K7" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L7" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="17" t="n">
+    <row r="8" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="28" t="n">
         <v>30026</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>10021</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="29" t="s">
         <v>55</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="I8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L8" s="12" t="b">
+      <c r="I8" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K8" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L8" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="26" t="n">
         <v>30027</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="29" t="s">
         <v>57</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="G9" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K9" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L9" s="12" t="b">
+      <c r="I9" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K9" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L9" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="26" t="n">
         <v>30028</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>10021</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="29" t="s">
         <v>59</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="I10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L10" s="12" t="b">
+      <c r="I10" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K10" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0" t="n">
+    <row r="11" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="28" t="n">
         <v>30029</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="29" t="s">
         <v>61</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="I11" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K11" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L11" s="12" t="b">
+      <c r="I11" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K11" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L11" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="26" t="n">
+    <row r="12" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="31" t="n">
         <v>30030</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="H12" s="0"/>
-      <c r="I12" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K12" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L12" s="12" t="b">
+      <c r="I12" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K12" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L12" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="n">
+    <row r="13" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="30" t="n">
         <v>30031</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="27" t="s">
+      <c r="F13" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="I13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K13" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L13" s="12" t="b">
+      <c r="I13" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K13" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L13" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="26" t="n">
+    <row r="14" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="31" t="n">
         <v>30032</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="G14" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="I14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L14" s="12" t="b">
+      <c r="I14" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K14" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L14" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17" t="n">
+    <row r="15" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="30" t="n">
         <v>30033</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="D15" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G15" s="27" t="s">
+      <c r="G15" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="I15" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K15" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L15" s="12" t="b">
+      <c r="I15" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K15" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L15" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="26" t="n">
+    <row r="16" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="31" t="n">
         <v>30034</v>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="G16" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="I16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L16" s="12" t="b">
+      <c r="I16" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K16" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L16" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="17" t="n">
+    <row r="17" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="30" t="n">
         <v>30035</v>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="I17" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L17" s="12" t="b">
+      <c r="I17" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K17" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L17" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="26" t="n">
+    <row r="18" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="31" t="n">
         <v>30036</v>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="I18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L18" s="12" t="b">
+      <c r="I18" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K18" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L18" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="n">
+    <row r="19" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="30" t="n">
         <v>30037</v>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="D19" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G19" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="I19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L19" s="12" t="b">
+      <c r="I19" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K19" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L19" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="0" t="n">
+    <row r="20" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="30" t="n">
         <v>30038</v>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D20" s="27" t="s">
+      <c r="D20" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E20" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G20" s="27" t="s">
+      <c r="G20" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="I20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K20" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L20" s="12" t="b">
+      <c r="I20" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K20" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L20" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="17" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -2083,7 +2125,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="17" width="11.01"/>
   </cols>
   <sheetData>
-    <row r="1" s="29" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2099,92 +2141,92 @@
       <c r="E1" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F1" s="28" t="n">
+      <c r="F1" s="34" t="n">
         <v>1</v>
       </c>
       <c r="G1" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="2" s="31" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="30" t="s">
+    <row r="2" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="36" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="32"/>
-      <c r="B3" s="33" t="n">
+      <c r="A3" s="38"/>
+      <c r="B3" s="39" t="n">
         <v>40021</v>
       </c>
-      <c r="C3" s="33" t="n">
+      <c r="C3" s="39" t="n">
         <v>30021</v>
       </c>
-      <c r="D3" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F3" s="34" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="G3" s="32"/>
+      <c r="D3" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="40" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G3" s="38"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35"/>
-      <c r="B4" s="34" t="n">
+      <c r="A4" s="41"/>
+      <c r="B4" s="40" t="n">
         <v>40022</v>
       </c>
-      <c r="C4" s="34" t="n">
+      <c r="C4" s="40" t="n">
         <v>30021</v>
       </c>
-      <c r="D4" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E4" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="34" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G4" s="35"/>
+      <c r="D4" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G4" s="41"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35"/>
-      <c r="B5" s="36" t="n">
+      <c r="A5" s="41"/>
+      <c r="B5" s="42" t="n">
         <v>40023</v>
       </c>
-      <c r="C5" s="36" t="n">
+      <c r="C5" s="42" t="n">
         <v>30021</v>
       </c>
-      <c r="D5" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E5" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F5" s="36" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G5" s="35"/>
+      <c r="D5" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F5" s="42" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G5" s="41"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="17" t="n">
@@ -2193,13 +2235,13 @@
       <c r="C6" s="17" t="n">
         <v>30022</v>
       </c>
-      <c r="D6" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F6" s="34" t="n">
+      <c r="D6" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F6" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2210,13 +2252,13 @@
       <c r="C7" s="17" t="n">
         <v>30022</v>
       </c>
-      <c r="D7" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E7" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="34" t="n">
+      <c r="D7" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2227,30 +2269,30 @@
       <c r="C8" s="17" t="n">
         <v>30022</v>
       </c>
-      <c r="D8" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E8" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F8" s="36" t="n">
+      <c r="D8" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F8" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="36" t="n">
+      <c r="B9" s="42" t="n">
         <v>40027</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>30023</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F9" s="34" t="n">
+      <c r="D9" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2261,13 +2303,13 @@
       <c r="C10" s="17" t="n">
         <v>30023</v>
       </c>
-      <c r="D10" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="34" t="n">
+      <c r="D10" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2278,64 +2320,64 @@
       <c r="C11" s="17" t="n">
         <v>30023</v>
       </c>
-      <c r="D11" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E11" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F11" s="36" t="n">
+      <c r="D11" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F11" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="33" t="n">
+      <c r="B12" s="39" t="n">
         <v>40030</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>30024</v>
       </c>
-      <c r="D12" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E12" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F12" s="34" t="n">
+      <c r="D12" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="34" t="n">
+      <c r="B13" s="40" t="n">
         <v>40031</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>30024</v>
       </c>
-      <c r="D13" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="34" t="n">
+      <c r="D13" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="36" t="n">
+      <c r="B14" s="42" t="n">
         <v>40032</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>30024</v>
       </c>
-      <c r="D14" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F14" s="36" t="n">
+      <c r="D14" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F14" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2346,13 +2388,13 @@
       <c r="C15" s="17" t="n">
         <v>30025</v>
       </c>
-      <c r="D15" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F15" s="34" t="n">
+      <c r="D15" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F15" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2363,13 +2405,13 @@
       <c r="C16" s="17" t="n">
         <v>30025</v>
       </c>
-      <c r="D16" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="34" t="n">
+      <c r="D16" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2380,30 +2422,30 @@
       <c r="C17" s="17" t="n">
         <v>30025</v>
       </c>
-      <c r="D17" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E17" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F17" s="36" t="n">
+      <c r="D17" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F17" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="36" t="n">
+      <c r="B18" s="42" t="n">
         <v>40036</v>
       </c>
       <c r="C18" s="17" t="n">
         <v>30026</v>
       </c>
-      <c r="D18" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E18" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F18" s="34" t="n">
+      <c r="D18" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F18" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2414,13 +2456,13 @@
       <c r="C19" s="17" t="n">
         <v>30026</v>
       </c>
-      <c r="D19" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="34" t="n">
+      <c r="D19" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2431,64 +2473,64 @@
       <c r="C20" s="17" t="n">
         <v>30026</v>
       </c>
-      <c r="D20" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F20" s="36" t="n">
+      <c r="D20" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F20" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="33" t="n">
+      <c r="B21" s="39" t="n">
         <v>40039</v>
       </c>
       <c r="C21" s="17" t="n">
         <v>30027</v>
       </c>
-      <c r="D21" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E21" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F21" s="34" t="n">
+      <c r="D21" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F21" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="34" t="n">
+      <c r="B22" s="40" t="n">
         <v>40040</v>
       </c>
       <c r="C22" s="17" t="n">
         <v>30027</v>
       </c>
-      <c r="D22" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="34" t="n">
+      <c r="D22" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="36" t="n">
+      <c r="B23" s="42" t="n">
         <v>40041</v>
       </c>
       <c r="C23" s="17" t="n">
         <v>30027</v>
       </c>
-      <c r="D23" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E23" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F23" s="36" t="n">
+      <c r="D23" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F23" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2499,13 +2541,13 @@
       <c r="C24" s="17" t="n">
         <v>30028</v>
       </c>
-      <c r="D24" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E24" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F24" s="34" t="n">
+      <c r="D24" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E24" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F24" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2516,13 +2558,13 @@
       <c r="C25" s="17" t="n">
         <v>30028</v>
       </c>
-      <c r="D25" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="34" t="n">
+      <c r="D25" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2533,64 +2575,64 @@
       <c r="C26" s="17" t="n">
         <v>30028</v>
       </c>
-      <c r="D26" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E26" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F26" s="36" t="n">
+      <c r="D26" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E26" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F26" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="33" t="n">
+      <c r="B27" s="39" t="n">
         <v>40045</v>
       </c>
       <c r="C27" s="17" t="n">
         <v>30029</v>
       </c>
-      <c r="D27" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E27" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F27" s="34" t="n">
+      <c r="D27" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E27" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F27" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="34" t="n">
+      <c r="B28" s="40" t="n">
         <v>40046</v>
       </c>
       <c r="C28" s="17" t="n">
         <v>30029</v>
       </c>
-      <c r="D28" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E28" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="34" t="n">
+      <c r="D28" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="36" t="n">
+      <c r="B29" s="42" t="n">
         <v>40047</v>
       </c>
       <c r="C29" s="17" t="n">
         <v>30029</v>
       </c>
-      <c r="D29" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E29" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F29" s="36" t="n">
+      <c r="D29" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F29" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2601,13 +2643,13 @@
       <c r="C30" s="17" t="n">
         <v>30030</v>
       </c>
-      <c r="D30" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E30" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F30" s="34" t="n">
+      <c r="D30" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F30" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2618,13 +2660,13 @@
       <c r="C31" s="17" t="n">
         <v>30030</v>
       </c>
-      <c r="D31" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="34" t="n">
+      <c r="D31" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E31" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2635,30 +2677,30 @@
       <c r="C32" s="17" t="n">
         <v>30030</v>
       </c>
-      <c r="D32" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F32" s="36" t="n">
+      <c r="D32" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F32" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="36" t="n">
+      <c r="B33" s="42" t="n">
         <v>40051</v>
       </c>
       <c r="C33" s="17" t="n">
         <v>30031</v>
       </c>
-      <c r="D33" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E33" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F33" s="34" t="n">
+      <c r="D33" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F33" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2669,13 +2711,13 @@
       <c r="C34" s="17" t="n">
         <v>30031</v>
       </c>
-      <c r="D34" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E34" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="34" t="n">
+      <c r="D34" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E34" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2686,64 +2728,64 @@
       <c r="C35" s="17" t="n">
         <v>30031</v>
       </c>
-      <c r="D35" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E35" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F35" s="36" t="n">
+      <c r="D35" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E35" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F35" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="33" t="n">
+      <c r="B36" s="39" t="n">
         <v>40054</v>
       </c>
       <c r="C36" s="17" t="n">
         <v>30032</v>
       </c>
-      <c r="D36" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E36" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F36" s="34" t="n">
+      <c r="D36" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E36" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F36" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="34" t="n">
+      <c r="B37" s="40" t="n">
         <v>40055</v>
       </c>
       <c r="C37" s="17" t="n">
         <v>30032</v>
       </c>
-      <c r="D37" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E37" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="34" t="n">
+      <c r="D37" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E37" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="36" t="n">
+      <c r="B38" s="42" t="n">
         <v>40056</v>
       </c>
       <c r="C38" s="17" t="n">
         <v>30032</v>
       </c>
-      <c r="D38" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E38" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F38" s="36" t="n">
+      <c r="D38" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E38" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F38" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2754,13 +2796,13 @@
       <c r="C39" s="17" t="n">
         <v>30033</v>
       </c>
-      <c r="D39" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E39" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F39" s="34" t="n">
+      <c r="D39" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E39" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F39" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2771,13 +2813,13 @@
       <c r="C40" s="17" t="n">
         <v>30033</v>
       </c>
-      <c r="D40" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E40" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="34" t="n">
+      <c r="D40" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E40" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2788,30 +2830,30 @@
       <c r="C41" s="17" t="n">
         <v>30033</v>
       </c>
-      <c r="D41" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E41" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F41" s="36" t="n">
+      <c r="D41" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F41" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="36" t="n">
+      <c r="B42" s="42" t="n">
         <v>40060</v>
       </c>
       <c r="C42" s="17" t="n">
         <v>30034</v>
       </c>
-      <c r="D42" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E42" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F42" s="34" t="n">
+      <c r="D42" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E42" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F42" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2822,13 +2864,13 @@
       <c r="C43" s="17" t="n">
         <v>30034</v>
       </c>
-      <c r="D43" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E43" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" s="34" t="n">
+      <c r="D43" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E43" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2839,64 +2881,64 @@
       <c r="C44" s="17" t="n">
         <v>30034</v>
       </c>
-      <c r="D44" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E44" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F44" s="36" t="n">
+      <c r="D44" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E44" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F44" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="33" t="n">
+      <c r="B45" s="39" t="n">
         <v>40063</v>
       </c>
       <c r="C45" s="17" t="n">
         <v>30035</v>
       </c>
-      <c r="D45" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E45" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F45" s="34" t="n">
+      <c r="D45" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E45" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F45" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="34" t="n">
+      <c r="B46" s="40" t="n">
         <v>40064</v>
       </c>
       <c r="C46" s="17" t="n">
         <v>30035</v>
       </c>
-      <c r="D46" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E46" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="34" t="n">
+      <c r="D46" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E46" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="36" t="n">
+      <c r="B47" s="42" t="n">
         <v>40065</v>
       </c>
       <c r="C47" s="17" t="n">
         <v>30035</v>
       </c>
-      <c r="D47" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E47" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F47" s="36" t="n">
+      <c r="D47" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E47" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F47" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2907,13 +2949,13 @@
       <c r="C48" s="17" t="n">
         <v>30036</v>
       </c>
-      <c r="D48" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E48" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F48" s="34" t="n">
+      <c r="D48" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E48" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F48" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2924,13 +2966,13 @@
       <c r="C49" s="17" t="n">
         <v>30036</v>
       </c>
-      <c r="D49" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E49" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" s="34" t="n">
+      <c r="D49" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E49" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2941,13 +2983,13 @@
       <c r="C50" s="17" t="n">
         <v>30036</v>
       </c>
-      <c r="D50" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E50" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F50" s="36" t="n">
+      <c r="D50" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E50" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F50" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2958,13 +3000,13 @@
       <c r="C51" s="17" t="n">
         <v>30037</v>
       </c>
-      <c r="D51" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E51" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F51" s="34" t="n">
+      <c r="D51" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E51" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F51" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2975,13 +3017,13 @@
       <c r="C52" s="17" t="n">
         <v>30037</v>
       </c>
-      <c r="D52" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E52" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="34" t="n">
+      <c r="D52" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E52" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2992,30 +3034,30 @@
       <c r="C53" s="17" t="n">
         <v>30037</v>
       </c>
-      <c r="D53" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E53" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F53" s="36" t="n">
+      <c r="D53" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E53" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F53" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="36" t="n">
+      <c r="B54" s="42" t="n">
         <v>40072</v>
       </c>
       <c r="C54" s="17" t="n">
         <v>30038</v>
       </c>
-      <c r="D54" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E54" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F54" s="34" t="n">
+      <c r="D54" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E54" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F54" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -3026,13 +3068,13 @@
       <c r="C55" s="17" t="n">
         <v>30038</v>
       </c>
-      <c r="D55" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E55" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="34" t="n">
+      <c r="D55" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E55" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -3043,13 +3085,13 @@
       <c r="C56" s="17" t="n">
         <v>30038</v>
       </c>
-      <c r="D56" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E56" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F56" s="36" t="n">
+      <c r="D56" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E56" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F56" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Features/skill lightattack default (#68)
* 플레이어에 CombatComponent 추가, EnemyBase->CharacterBase 변경 중

* 기본공격 1, 공격 시 이동 잠금 상태 추가

* PlayerState 추가
히트스윕 시각화 설정

* 무기 소켓 설정

- 무기 애셋에 Sword_Start, Sword_End 소켓 설정
- CharacterBase에 무기 메쉬 가상 함수 추가
- CombatComponent에서 Owner에 무기 메쉬가 있을 경우 무기 메쉬에서 소켓 탐색

* 기본공격 1, 종료 노티파이 추가
</commit_message>
<xml_diff>
--- a/BADesign/Excel/Action.xlsx
+++ b/BADesign/Excel/Action.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ActionData" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="80">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t xml:space="preserve">/Game/Character/Player/Animation/Montages/DodgeRoll/AM_Dodge_Relaxed_BackwardRight.AM_Dodge_Relaxed_BackwardRight</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">ActionAnimationTid</t>
@@ -326,7 +329,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -342,7 +345,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFFFF5CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFD7"/>
+        <bgColor rgb="FFFFF5CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF5CE"/>
+        <bgColor rgb="FFFFFFD7"/>
       </patternFill>
     </fill>
   </fills>
@@ -380,7 +395,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -481,15 +496,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -558,7 +597,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFFFD7"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -575,7 +614,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFF5CE"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -1366,8 +1405,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultColWidth="7.6875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L22"/>
+  <sheetFormatPr defaultColWidth="7.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="9.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="14.38"/>
@@ -1457,7 +1496,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25"/>
       <c r="B3" s="25" t="n">
         <v>30021</v>
@@ -1471,588 +1510,591 @@
       <c r="E3" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="27" t="s">
         <v>39</v>
       </c>
       <c r="G3" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L3" s="12" t="b">
+      <c r="H3" s="27"/>
+      <c r="I3" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K3" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L3" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="n">
+    <row r="4" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="28" t="n">
         <v>30022</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="28" t="s">
         <v>48</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="27" t="s">
         <v>39</v>
       </c>
       <c r="G4" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="0"/>
-      <c r="I4" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L4" s="12" t="b">
+      <c r="I4" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K4" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L4" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="17" t="n">
+    <row r="5" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="28" t="n">
         <v>30023</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="27" t="s">
         <v>49</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G5" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K5" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L5" s="12" t="b">
+      <c r="I5" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K5" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L5" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="17" t="n">
+    <row r="6" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="28" t="n">
         <v>30024</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>10021</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="D6" s="29" t="s">
         <v>51</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="I6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L6" s="12" t="b">
+      <c r="I6" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K6" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L6" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="26" t="n">
         <v>30025</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" s="29" t="s">
         <v>53</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G7" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="I7" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K7" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L7" s="12" t="b">
+      <c r="I7" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K7" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L7" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="17" t="n">
+    <row r="8" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="28" t="n">
         <v>30026</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>10021</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="29" t="s">
         <v>55</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="I8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L8" s="12" t="b">
+      <c r="I8" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K8" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L8" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="26" t="n">
         <v>30027</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="29" t="s">
         <v>57</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="G9" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K9" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L9" s="12" t="b">
+      <c r="I9" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K9" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L9" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="26" t="n">
         <v>30028</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>10021</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="29" t="s">
         <v>59</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="I10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L10" s="12" t="b">
+      <c r="I10" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K10" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0" t="n">
+    <row r="11" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="28" t="n">
         <v>30029</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="28" t="n">
         <v>10021</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="29" t="s">
         <v>61</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="I11" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K11" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L11" s="12" t="b">
+      <c r="I11" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K11" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L11" s="27" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="26" t="n">
+    <row r="12" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="31" t="n">
         <v>30030</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="H12" s="0"/>
-      <c r="I12" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K12" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L12" s="12" t="b">
+      <c r="I12" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K12" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L12" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="n">
+    <row r="13" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="30" t="n">
         <v>30031</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="27" t="s">
+      <c r="F13" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="I13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K13" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L13" s="12" t="b">
+      <c r="I13" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K13" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L13" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="26" t="n">
+    <row r="14" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="31" t="n">
         <v>30032</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="G14" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="I14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L14" s="12" t="b">
+      <c r="I14" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K14" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L14" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17" t="n">
+    <row r="15" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="30" t="n">
         <v>30033</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="D15" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G15" s="27" t="s">
+      <c r="G15" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="I15" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K15" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L15" s="12" t="b">
+      <c r="I15" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K15" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L15" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="26" t="n">
+    <row r="16" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="31" t="n">
         <v>30034</v>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="G16" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="I16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L16" s="12" t="b">
+      <c r="I16" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K16" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L16" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="17" t="n">
+    <row r="17" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="30" t="n">
         <v>30035</v>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="I17" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L17" s="12" t="b">
+      <c r="I17" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K17" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L17" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="26" t="n">
+    <row r="18" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="31" t="n">
         <v>30036</v>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="I18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L18" s="12" t="b">
+      <c r="I18" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K18" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L18" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="n">
+    <row r="19" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="30" t="n">
         <v>30037</v>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="D19" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G19" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="I19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L19" s="12" t="b">
+      <c r="I19" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K19" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L19" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="0" t="n">
+    <row r="20" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="30" t="n">
         <v>30038</v>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="30" t="n">
         <v>10022</v>
       </c>
-      <c r="D20" s="27" t="s">
+      <c r="D20" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E20" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G20" s="27" t="s">
+      <c r="G20" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="I20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K20" s="12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L20" s="12" t="b">
+      <c r="I20" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K20" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L20" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="17" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -2083,7 +2125,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="17" width="11.01"/>
   </cols>
   <sheetData>
-    <row r="1" s="29" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2099,92 +2141,92 @@
       <c r="E1" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F1" s="28" t="n">
+      <c r="F1" s="34" t="n">
         <v>1</v>
       </c>
       <c r="G1" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="2" s="31" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="30" t="s">
+    <row r="2" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="36" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="32"/>
-      <c r="B3" s="33" t="n">
+      <c r="A3" s="38"/>
+      <c r="B3" s="39" t="n">
         <v>40021</v>
       </c>
-      <c r="C3" s="33" t="n">
+      <c r="C3" s="39" t="n">
         <v>30021</v>
       </c>
-      <c r="D3" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F3" s="34" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="G3" s="32"/>
+      <c r="D3" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="40" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G3" s="38"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35"/>
-      <c r="B4" s="34" t="n">
+      <c r="A4" s="41"/>
+      <c r="B4" s="40" t="n">
         <v>40022</v>
       </c>
-      <c r="C4" s="34" t="n">
+      <c r="C4" s="40" t="n">
         <v>30021</v>
       </c>
-      <c r="D4" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E4" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="34" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G4" s="35"/>
+      <c r="D4" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G4" s="41"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35"/>
-      <c r="B5" s="36" t="n">
+      <c r="A5" s="41"/>
+      <c r="B5" s="42" t="n">
         <v>40023</v>
       </c>
-      <c r="C5" s="36" t="n">
+      <c r="C5" s="42" t="n">
         <v>30021</v>
       </c>
-      <c r="D5" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E5" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F5" s="36" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G5" s="35"/>
+      <c r="D5" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F5" s="42" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G5" s="41"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="17" t="n">
@@ -2193,13 +2235,13 @@
       <c r="C6" s="17" t="n">
         <v>30022</v>
       </c>
-      <c r="D6" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F6" s="34" t="n">
+      <c r="D6" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F6" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2210,13 +2252,13 @@
       <c r="C7" s="17" t="n">
         <v>30022</v>
       </c>
-      <c r="D7" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E7" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="34" t="n">
+      <c r="D7" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2227,30 +2269,30 @@
       <c r="C8" s="17" t="n">
         <v>30022</v>
       </c>
-      <c r="D8" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E8" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F8" s="36" t="n">
+      <c r="D8" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F8" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="36" t="n">
+      <c r="B9" s="42" t="n">
         <v>40027</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>30023</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F9" s="34" t="n">
+      <c r="D9" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2261,13 +2303,13 @@
       <c r="C10" s="17" t="n">
         <v>30023</v>
       </c>
-      <c r="D10" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="34" t="n">
+      <c r="D10" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2278,64 +2320,64 @@
       <c r="C11" s="17" t="n">
         <v>30023</v>
       </c>
-      <c r="D11" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E11" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F11" s="36" t="n">
+      <c r="D11" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F11" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="33" t="n">
+      <c r="B12" s="39" t="n">
         <v>40030</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>30024</v>
       </c>
-      <c r="D12" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E12" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F12" s="34" t="n">
+      <c r="D12" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="34" t="n">
+      <c r="B13" s="40" t="n">
         <v>40031</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>30024</v>
       </c>
-      <c r="D13" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="34" t="n">
+      <c r="D13" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="36" t="n">
+      <c r="B14" s="42" t="n">
         <v>40032</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>30024</v>
       </c>
-      <c r="D14" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F14" s="36" t="n">
+      <c r="D14" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F14" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2346,13 +2388,13 @@
       <c r="C15" s="17" t="n">
         <v>30025</v>
       </c>
-      <c r="D15" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F15" s="34" t="n">
+      <c r="D15" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F15" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2363,13 +2405,13 @@
       <c r="C16" s="17" t="n">
         <v>30025</v>
       </c>
-      <c r="D16" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="34" t="n">
+      <c r="D16" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2380,30 +2422,30 @@
       <c r="C17" s="17" t="n">
         <v>30025</v>
       </c>
-      <c r="D17" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E17" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F17" s="36" t="n">
+      <c r="D17" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F17" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="36" t="n">
+      <c r="B18" s="42" t="n">
         <v>40036</v>
       </c>
       <c r="C18" s="17" t="n">
         <v>30026</v>
       </c>
-      <c r="D18" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E18" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F18" s="34" t="n">
+      <c r="D18" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F18" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2414,13 +2456,13 @@
       <c r="C19" s="17" t="n">
         <v>30026</v>
       </c>
-      <c r="D19" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="34" t="n">
+      <c r="D19" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2431,64 +2473,64 @@
       <c r="C20" s="17" t="n">
         <v>30026</v>
       </c>
-      <c r="D20" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F20" s="36" t="n">
+      <c r="D20" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F20" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="33" t="n">
+      <c r="B21" s="39" t="n">
         <v>40039</v>
       </c>
       <c r="C21" s="17" t="n">
         <v>30027</v>
       </c>
-      <c r="D21" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E21" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F21" s="34" t="n">
+      <c r="D21" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F21" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="34" t="n">
+      <c r="B22" s="40" t="n">
         <v>40040</v>
       </c>
       <c r="C22" s="17" t="n">
         <v>30027</v>
       </c>
-      <c r="D22" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="34" t="n">
+      <c r="D22" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="36" t="n">
+      <c r="B23" s="42" t="n">
         <v>40041</v>
       </c>
       <c r="C23" s="17" t="n">
         <v>30027</v>
       </c>
-      <c r="D23" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E23" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F23" s="36" t="n">
+      <c r="D23" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F23" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2499,13 +2541,13 @@
       <c r="C24" s="17" t="n">
         <v>30028</v>
       </c>
-      <c r="D24" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E24" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F24" s="34" t="n">
+      <c r="D24" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E24" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F24" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2516,13 +2558,13 @@
       <c r="C25" s="17" t="n">
         <v>30028</v>
       </c>
-      <c r="D25" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="34" t="n">
+      <c r="D25" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2533,64 +2575,64 @@
       <c r="C26" s="17" t="n">
         <v>30028</v>
       </c>
-      <c r="D26" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E26" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F26" s="36" t="n">
+      <c r="D26" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E26" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F26" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="33" t="n">
+      <c r="B27" s="39" t="n">
         <v>40045</v>
       </c>
       <c r="C27" s="17" t="n">
         <v>30029</v>
       </c>
-      <c r="D27" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E27" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F27" s="34" t="n">
+      <c r="D27" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E27" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F27" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="34" t="n">
+      <c r="B28" s="40" t="n">
         <v>40046</v>
       </c>
       <c r="C28" s="17" t="n">
         <v>30029</v>
       </c>
-      <c r="D28" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E28" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="34" t="n">
+      <c r="D28" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="36" t="n">
+      <c r="B29" s="42" t="n">
         <v>40047</v>
       </c>
       <c r="C29" s="17" t="n">
         <v>30029</v>
       </c>
-      <c r="D29" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E29" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F29" s="36" t="n">
+      <c r="D29" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F29" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2601,13 +2643,13 @@
       <c r="C30" s="17" t="n">
         <v>30030</v>
       </c>
-      <c r="D30" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E30" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F30" s="34" t="n">
+      <c r="D30" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F30" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2618,13 +2660,13 @@
       <c r="C31" s="17" t="n">
         <v>30030</v>
       </c>
-      <c r="D31" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="34" t="n">
+      <c r="D31" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E31" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2635,30 +2677,30 @@
       <c r="C32" s="17" t="n">
         <v>30030</v>
       </c>
-      <c r="D32" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F32" s="36" t="n">
+      <c r="D32" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F32" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="36" t="n">
+      <c r="B33" s="42" t="n">
         <v>40051</v>
       </c>
       <c r="C33" s="17" t="n">
         <v>30031</v>
       </c>
-      <c r="D33" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E33" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F33" s="34" t="n">
+      <c r="D33" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F33" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2669,13 +2711,13 @@
       <c r="C34" s="17" t="n">
         <v>30031</v>
       </c>
-      <c r="D34" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E34" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="34" t="n">
+      <c r="D34" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E34" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2686,64 +2728,64 @@
       <c r="C35" s="17" t="n">
         <v>30031</v>
       </c>
-      <c r="D35" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E35" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F35" s="36" t="n">
+      <c r="D35" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E35" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F35" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="33" t="n">
+      <c r="B36" s="39" t="n">
         <v>40054</v>
       </c>
       <c r="C36" s="17" t="n">
         <v>30032</v>
       </c>
-      <c r="D36" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E36" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F36" s="34" t="n">
+      <c r="D36" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E36" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F36" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="34" t="n">
+      <c r="B37" s="40" t="n">
         <v>40055</v>
       </c>
       <c r="C37" s="17" t="n">
         <v>30032</v>
       </c>
-      <c r="D37" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E37" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="34" t="n">
+      <c r="D37" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E37" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="36" t="n">
+      <c r="B38" s="42" t="n">
         <v>40056</v>
       </c>
       <c r="C38" s="17" t="n">
         <v>30032</v>
       </c>
-      <c r="D38" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E38" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F38" s="36" t="n">
+      <c r="D38" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E38" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F38" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2754,13 +2796,13 @@
       <c r="C39" s="17" t="n">
         <v>30033</v>
       </c>
-      <c r="D39" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E39" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F39" s="34" t="n">
+      <c r="D39" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E39" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F39" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2771,13 +2813,13 @@
       <c r="C40" s="17" t="n">
         <v>30033</v>
       </c>
-      <c r="D40" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E40" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="34" t="n">
+      <c r="D40" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E40" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2788,30 +2830,30 @@
       <c r="C41" s="17" t="n">
         <v>30033</v>
       </c>
-      <c r="D41" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E41" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F41" s="36" t="n">
+      <c r="D41" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F41" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="36" t="n">
+      <c r="B42" s="42" t="n">
         <v>40060</v>
       </c>
       <c r="C42" s="17" t="n">
         <v>30034</v>
       </c>
-      <c r="D42" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E42" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F42" s="34" t="n">
+      <c r="D42" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E42" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F42" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2822,13 +2864,13 @@
       <c r="C43" s="17" t="n">
         <v>30034</v>
       </c>
-      <c r="D43" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E43" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" s="34" t="n">
+      <c r="D43" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E43" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2839,64 +2881,64 @@
       <c r="C44" s="17" t="n">
         <v>30034</v>
       </c>
-      <c r="D44" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E44" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F44" s="36" t="n">
+      <c r="D44" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E44" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F44" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="33" t="n">
+      <c r="B45" s="39" t="n">
         <v>40063</v>
       </c>
       <c r="C45" s="17" t="n">
         <v>30035</v>
       </c>
-      <c r="D45" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E45" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F45" s="34" t="n">
+      <c r="D45" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E45" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F45" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="34" t="n">
+      <c r="B46" s="40" t="n">
         <v>40064</v>
       </c>
       <c r="C46" s="17" t="n">
         <v>30035</v>
       </c>
-      <c r="D46" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E46" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="34" t="n">
+      <c r="D46" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E46" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="36" t="n">
+      <c r="B47" s="42" t="n">
         <v>40065</v>
       </c>
       <c r="C47" s="17" t="n">
         <v>30035</v>
       </c>
-      <c r="D47" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E47" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F47" s="36" t="n">
+      <c r="D47" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E47" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F47" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2907,13 +2949,13 @@
       <c r="C48" s="17" t="n">
         <v>30036</v>
       </c>
-      <c r="D48" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E48" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F48" s="34" t="n">
+      <c r="D48" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E48" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F48" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2924,13 +2966,13 @@
       <c r="C49" s="17" t="n">
         <v>30036</v>
       </c>
-      <c r="D49" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E49" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" s="34" t="n">
+      <c r="D49" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E49" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2941,13 +2983,13 @@
       <c r="C50" s="17" t="n">
         <v>30036</v>
       </c>
-      <c r="D50" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E50" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F50" s="36" t="n">
+      <c r="D50" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E50" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F50" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2958,13 +3000,13 @@
       <c r="C51" s="17" t="n">
         <v>30037</v>
       </c>
-      <c r="D51" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E51" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F51" s="34" t="n">
+      <c r="D51" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E51" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F51" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2975,13 +3017,13 @@
       <c r="C52" s="17" t="n">
         <v>30037</v>
       </c>
-      <c r="D52" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E52" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="34" t="n">
+      <c r="D52" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E52" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -2992,30 +3034,30 @@
       <c r="C53" s="17" t="n">
         <v>30037</v>
       </c>
-      <c r="D53" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E53" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F53" s="36" t="n">
+      <c r="D53" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E53" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F53" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="36" t="n">
+      <c r="B54" s="42" t="n">
         <v>40072</v>
       </c>
       <c r="C54" s="17" t="n">
         <v>30038</v>
       </c>
-      <c r="D54" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E54" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F54" s="34" t="n">
+      <c r="D54" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E54" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F54" s="40" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -3026,13 +3068,13 @@
       <c r="C55" s="17" t="n">
         <v>30038</v>
       </c>
-      <c r="D55" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E55" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="34" t="n">
+      <c r="D55" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E55" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="40" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -3043,13 +3085,13 @@
       <c r="C56" s="17" t="n">
         <v>30038</v>
       </c>
-      <c r="D56" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E56" s="36" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F56" s="36" t="n">
+      <c r="D56" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="E56" s="42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F56" s="42" t="n">
         <v>0.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Features/skill lightattack default (#70)
* 플레이어에 CombatComponent 추가, EnemyBase->CharacterBase 변경 중

* 기본공격 1, 공격 시 이동 잠금 상태 추가

* PlayerState 추가
히트스윕 시각화 설정

* 무기 소켓 설정

- 무기 애셋에 Sword_Start, Sword_End 소켓 설정
- CharacterBase에 무기 메쉬 가상 함수 추가
- CombatComponent에서 Owner에 무기 메쉬가 있을 경우 무기 메쉬에서 소켓 탐색

* 기본공격 1, 종료 노티파이 추가

* Great_Sword 추가(Socket 추가됨)
콤보 로직 작성 중

* 좌좌 콤보 구현

* 회피 타이밍 갱신
</commit_message>
<xml_diff>
--- a/BADesign/Excel/Action.xlsx
+++ b/BADesign/Excel/Action.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="85">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -166,6 +166,9 @@
     <t xml:space="preserve">bUseRootMotion</t>
   </si>
   <si>
+    <t xml:space="preserve">NextComboLAnimationTid</t>
+  </si>
+  <si>
     <t xml:space="preserve">/Game/Character/Player/Animation/Montages/DodgeRoll/AM_Roll_Relaxed_Forward.AM_Roll_Relaxed_Forward</t>
   </si>
   <si>
@@ -238,7 +241,19 @@
     <t xml:space="preserve">/Game/Character/Player/Animation/Montages/DodgeRoll/AM_Dodge_Relaxed_BackwardRight.AM_Dodge_Relaxed_BackwardRight</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t xml:space="preserve">/Game/Character/Player/Animation/Montages/LightAttack/AM_Player_LightAttack_1.AM_Player_LightAttack_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기본공격1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Character/Player/Animation/Montages/LightAttack/AM_Player_LightAttack_2.AM_Player_LightAttack_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기본공격2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">강공격1</t>
   </si>
   <si>
     <t xml:space="preserve">ActionAnimationTid</t>
@@ -492,7 +507,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1405,7 +1420,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr defaultColWidth="7.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="9.3"/>
@@ -1417,7 +1432,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="17" width="12.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="17" width="11.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="17" width="10.87"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="13" style="17" width="7.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="17" width="17.96"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="14" style="17" width="7.68"/>
   </cols>
   <sheetData>
     <row r="1" s="20" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1457,6 +1473,12 @@
       <c r="L1" s="19" t="n">
         <v>1</v>
       </c>
+      <c r="M1" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="2" s="24" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
@@ -1494,6 +1516,9 @@
       </c>
       <c r="L2" s="23" t="s">
         <v>46</v>
+      </c>
+      <c r="M2" s="24" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="3" s="28" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1514,7 +1539,7 @@
         <v>39</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H3" s="27"/>
       <c r="I3" s="27" t="n">
@@ -1539,7 +1564,7 @@
         <v>10021</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>37</v>
@@ -1548,7 +1573,7 @@
         <v>39</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I4" s="27" t="n">
         <v>1</v>
@@ -1572,7 +1597,7 @@
         <v>10021</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>37</v>
@@ -1581,7 +1606,7 @@
         <v>39</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I5" s="28" t="n">
         <v>1</v>
@@ -1605,7 +1630,7 @@
         <v>10021</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>37</v>
@@ -1614,7 +1639,7 @@
         <v>39</v>
       </c>
       <c r="G6" s="29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I6" s="27" t="n">
         <v>1</v>
@@ -1638,7 +1663,7 @@
         <v>10021</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>37</v>
@@ -1647,7 +1672,7 @@
         <v>39</v>
       </c>
       <c r="G7" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I7" s="28" t="n">
         <v>1</v>
@@ -1671,7 +1696,7 @@
         <v>10021</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>37</v>
@@ -1680,7 +1705,7 @@
         <v>39</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I8" s="27" t="n">
         <v>1</v>
@@ -1704,7 +1729,7 @@
         <v>10021</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>37</v>
@@ -1713,7 +1738,7 @@
         <v>39</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I9" s="28" t="n">
         <v>1</v>
@@ -1737,7 +1762,7 @@
         <v>10021</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>37</v>
@@ -1746,7 +1771,7 @@
         <v>39</v>
       </c>
       <c r="G10" s="29" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I10" s="27" t="n">
         <v>1</v>
@@ -1770,7 +1795,7 @@
         <v>10021</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>37</v>
@@ -1779,7 +1804,7 @@
         <v>39</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I11" s="28" t="n">
         <v>1</v>
@@ -1812,7 +1837,7 @@
         <v>39</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I12" s="30" t="n">
         <v>1</v>
@@ -1836,7 +1861,7 @@
         <v>10022</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E13" s="33" t="s">
         <v>37</v>
@@ -1845,7 +1870,7 @@
         <v>39</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I13" s="30" t="n">
         <v>1</v>
@@ -1869,7 +1894,7 @@
         <v>10022</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" s="31" t="s">
         <v>37</v>
@@ -1878,7 +1903,7 @@
         <v>39</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I14" s="32" t="n">
         <v>1</v>
@@ -1902,7 +1927,7 @@
         <v>10022</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="31" t="s">
         <v>37</v>
@@ -1911,7 +1936,7 @@
         <v>39</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I15" s="30" t="n">
         <v>1</v>
@@ -1935,7 +1960,7 @@
         <v>10022</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E16" s="31" t="s">
         <v>37</v>
@@ -1944,7 +1969,7 @@
         <v>39</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I16" s="32" t="n">
         <v>1</v>
@@ -1968,7 +1993,7 @@
         <v>10022</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E17" s="31" t="s">
         <v>37</v>
@@ -1977,7 +2002,7 @@
         <v>39</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I17" s="30" t="n">
         <v>1</v>
@@ -2001,7 +2026,7 @@
         <v>10022</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>37</v>
@@ -2010,7 +2035,7 @@
         <v>39</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I18" s="32" t="n">
         <v>1</v>
@@ -2034,7 +2059,7 @@
         <v>10022</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E19" s="31" t="s">
         <v>37</v>
@@ -2043,7 +2068,7 @@
         <v>39</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I19" s="30" t="n">
         <v>1</v>
@@ -2067,7 +2092,7 @@
         <v>10022</v>
       </c>
       <c r="D20" s="33" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E20" s="31" t="s">
         <v>37</v>
@@ -2076,7 +2101,7 @@
         <v>39</v>
       </c>
       <c r="G20" s="33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I20" s="32" t="n">
         <v>1</v>
@@ -2092,9 +2117,37 @@
         <v>1</v>
       </c>
     </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="17" t="n">
+        <v>31001</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="M21" s="17" t="n">
+        <v>31002</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>73</v>
+      </c>
+    </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="17" t="s">
-        <v>71</v>
+      <c r="B22" s="17" t="n">
+        <v>31002</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="17" t="n">
+        <v>32001</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2156,19 +2209,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2180,7 +2233,7 @@
         <v>30021</v>
       </c>
       <c r="D3" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E3" s="39" t="n">
         <v>0.1</v>
@@ -2199,7 +2252,7 @@
         <v>30021</v>
       </c>
       <c r="D4" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E4" s="40" t="n">
         <v>0</v>
@@ -2218,7 +2271,7 @@
         <v>30021</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E5" s="42" t="n">
         <v>0.55</v>
@@ -2236,7 +2289,7 @@
         <v>30022</v>
       </c>
       <c r="D6" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>0.1</v>
@@ -2253,7 +2306,7 @@
         <v>30022</v>
       </c>
       <c r="D7" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E7" s="40" t="n">
         <v>0</v>
@@ -2270,7 +2323,7 @@
         <v>30022</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E8" s="42" t="n">
         <v>0.55</v>
@@ -2287,7 +2340,7 @@
         <v>30023</v>
       </c>
       <c r="D9" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E9" s="39" t="n">
         <v>0.1</v>
@@ -2304,7 +2357,7 @@
         <v>30023</v>
       </c>
       <c r="D10" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E10" s="40" t="n">
         <v>0</v>
@@ -2321,7 +2374,7 @@
         <v>30023</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E11" s="42" t="n">
         <v>0.55</v>
@@ -2338,7 +2391,7 @@
         <v>30024</v>
       </c>
       <c r="D12" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E12" s="39" t="n">
         <v>0.1</v>
@@ -2355,7 +2408,7 @@
         <v>30024</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E13" s="40" t="n">
         <v>0</v>
@@ -2372,7 +2425,7 @@
         <v>30024</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E14" s="42" t="n">
         <v>0.55</v>
@@ -2389,7 +2442,7 @@
         <v>30025</v>
       </c>
       <c r="D15" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E15" s="39" t="n">
         <v>0.1</v>
@@ -2406,7 +2459,7 @@
         <v>30025</v>
       </c>
       <c r="D16" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E16" s="40" t="n">
         <v>0</v>
@@ -2423,7 +2476,7 @@
         <v>30025</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E17" s="42" t="n">
         <v>0.55</v>
@@ -2440,7 +2493,7 @@
         <v>30026</v>
       </c>
       <c r="D18" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E18" s="39" t="n">
         <v>0.1</v>
@@ -2457,7 +2510,7 @@
         <v>30026</v>
       </c>
       <c r="D19" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E19" s="40" t="n">
         <v>0</v>
@@ -2474,7 +2527,7 @@
         <v>30026</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E20" s="42" t="n">
         <v>0.55</v>
@@ -2491,7 +2544,7 @@
         <v>30027</v>
       </c>
       <c r="D21" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E21" s="39" t="n">
         <v>0.1</v>
@@ -2508,7 +2561,7 @@
         <v>30027</v>
       </c>
       <c r="D22" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E22" s="40" t="n">
         <v>0</v>
@@ -2525,7 +2578,7 @@
         <v>30027</v>
       </c>
       <c r="D23" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E23" s="42" t="n">
         <v>0.55</v>
@@ -2542,7 +2595,7 @@
         <v>30028</v>
       </c>
       <c r="D24" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E24" s="39" t="n">
         <v>0.1</v>
@@ -2559,7 +2612,7 @@
         <v>30028</v>
       </c>
       <c r="D25" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E25" s="40" t="n">
         <v>0</v>
@@ -2576,7 +2629,7 @@
         <v>30028</v>
       </c>
       <c r="D26" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E26" s="42" t="n">
         <v>0.55</v>
@@ -2593,7 +2646,7 @@
         <v>30029</v>
       </c>
       <c r="D27" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E27" s="39" t="n">
         <v>0.1</v>
@@ -2610,7 +2663,7 @@
         <v>30029</v>
       </c>
       <c r="D28" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E28" s="40" t="n">
         <v>0</v>
@@ -2627,7 +2680,7 @@
         <v>30029</v>
       </c>
       <c r="D29" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E29" s="42" t="n">
         <v>0.55</v>
@@ -2644,7 +2697,7 @@
         <v>30030</v>
       </c>
       <c r="D30" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E30" s="39" t="n">
         <v>0.1</v>
@@ -2661,7 +2714,7 @@
         <v>30030</v>
       </c>
       <c r="D31" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E31" s="40" t="n">
         <v>0</v>
@@ -2678,7 +2731,7 @@
         <v>30030</v>
       </c>
       <c r="D32" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E32" s="42" t="n">
         <v>0.55</v>
@@ -2695,7 +2748,7 @@
         <v>30031</v>
       </c>
       <c r="D33" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E33" s="39" t="n">
         <v>0.1</v>
@@ -2712,7 +2765,7 @@
         <v>30031</v>
       </c>
       <c r="D34" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E34" s="40" t="n">
         <v>0</v>
@@ -2729,7 +2782,7 @@
         <v>30031</v>
       </c>
       <c r="D35" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E35" s="42" t="n">
         <v>0.55</v>
@@ -2746,7 +2799,7 @@
         <v>30032</v>
       </c>
       <c r="D36" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E36" s="39" t="n">
         <v>0.1</v>
@@ -2763,7 +2816,7 @@
         <v>30032</v>
       </c>
       <c r="D37" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E37" s="40" t="n">
         <v>0</v>
@@ -2780,7 +2833,7 @@
         <v>30032</v>
       </c>
       <c r="D38" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E38" s="42" t="n">
         <v>0.55</v>
@@ -2797,7 +2850,7 @@
         <v>30033</v>
       </c>
       <c r="D39" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E39" s="39" t="n">
         <v>0.1</v>
@@ -2814,7 +2867,7 @@
         <v>30033</v>
       </c>
       <c r="D40" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E40" s="40" t="n">
         <v>0</v>
@@ -2831,7 +2884,7 @@
         <v>30033</v>
       </c>
       <c r="D41" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E41" s="42" t="n">
         <v>0.55</v>
@@ -2848,7 +2901,7 @@
         <v>30034</v>
       </c>
       <c r="D42" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E42" s="39" t="n">
         <v>0.1</v>
@@ -2865,7 +2918,7 @@
         <v>30034</v>
       </c>
       <c r="D43" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E43" s="40" t="n">
         <v>0</v>
@@ -2882,7 +2935,7 @@
         <v>30034</v>
       </c>
       <c r="D44" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E44" s="42" t="n">
         <v>0.55</v>
@@ -2899,7 +2952,7 @@
         <v>30035</v>
       </c>
       <c r="D45" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E45" s="39" t="n">
         <v>0.1</v>
@@ -2916,7 +2969,7 @@
         <v>30035</v>
       </c>
       <c r="D46" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E46" s="40" t="n">
         <v>0</v>
@@ -2933,7 +2986,7 @@
         <v>30035</v>
       </c>
       <c r="D47" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E47" s="42" t="n">
         <v>0.55</v>
@@ -2950,7 +3003,7 @@
         <v>30036</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E48" s="39" t="n">
         <v>0.1</v>
@@ -2967,7 +3020,7 @@
         <v>30036</v>
       </c>
       <c r="D49" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E49" s="40" t="n">
         <v>0</v>
@@ -2984,7 +3037,7 @@
         <v>30036</v>
       </c>
       <c r="D50" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E50" s="42" t="n">
         <v>0.55</v>
@@ -3001,7 +3054,7 @@
         <v>30037</v>
       </c>
       <c r="D51" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E51" s="39" t="n">
         <v>0.1</v>
@@ -3018,7 +3071,7 @@
         <v>30037</v>
       </c>
       <c r="D52" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E52" s="40" t="n">
         <v>0</v>
@@ -3035,7 +3088,7 @@
         <v>30037</v>
       </c>
       <c r="D53" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E53" s="42" t="n">
         <v>0.55</v>
@@ -3052,7 +3105,7 @@
         <v>30038</v>
       </c>
       <c r="D54" s="39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E54" s="39" t="n">
         <v>0.1</v>
@@ -3069,7 +3122,7 @@
         <v>30038</v>
       </c>
       <c r="D55" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E55" s="40" t="n">
         <v>0</v>
@@ -3086,7 +3139,7 @@
         <v>30038</v>
       </c>
       <c r="D56" s="42" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E56" s="42" t="n">
         <v>0.55</v>

</xml_diff>

<commit_message>
Features/skill apply action (#108)
* 캐릭터 콤보 변경 함수 작성

* 강공격 기본값 오버라이드 삭제

* 컴파일 오류 수정

* 콤보 오버라이드 로직 완성, 강공격 기본값 수정

- 차징공격 스킬 찍으면 강공격이 차징공격으로 바뀝니다.

* 첫 공격 엑셀 테이블에서 지정하도록 수정

* LRR 커맨드 스킬 추가..

* 콤보 관련 스킬 추가

* 플레이어 속성 공격 트레일 vfx 수정
</commit_message>
<xml_diff>
--- a/BADesign/Excel/Action.xlsx
+++ b/BADesign/Excel/Action.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="110">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -281,15 +281,15 @@
     <t xml:space="preserve">DamageCoefficient</t>
   </si>
   <si>
+    <t xml:space="preserve">시작 공격 지정</t>
+  </si>
+  <si>
     <t xml:space="preserve">기본공격1</t>
   </si>
   <si>
     <t xml:space="preserve">/Game/Character/Player/Animation/Montages/LightAttack/AM_Player_LightAttack_1.AM_Player_LightAttack_1</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t xml:space="preserve">기본공격2</t>
   </si>
   <si>
@@ -330,6 +330,30 @@
   </si>
   <si>
     <t xml:space="preserve">/Game/Character/Player/Animation/Montages/HeavyAttack/AM_Player_ChargeAttack.AM_Player_ChargeAttack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L”R”R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Character/Player/Animation/Montages/HeavyAttack/AM_Player_HeavyAttack_3.AM_Player_HeavyAttack_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR”R”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Character/Player/Animation/Montages/HeavyAttack/AM_Player_HeavyAttack_4.AM_Player_HeavyAttack_4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">좀 더 큰 강공격</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Character/Player/Animation/Montages/HeavyAttack/AM_Player_HeavyAttack_5.AM_Player_HeavyAttack_5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기본공격4 대체 – 위로 띄우는 공격</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Character/Player/Animation/Montages/LightAttack/AM_Player_LightAttack_5.AM_Player_LightAttack_5</t>
   </si>
 </sst>
 </file>
@@ -350,19 +374,16 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="12"/>
@@ -489,127 +510,127 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -713,37 +734,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285f4"/>
+        <a:srgbClr val="4285F4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ea4335"/>
+        <a:srgbClr val="EA4335"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="fbbc04"/>
+        <a:srgbClr val="FBBC04"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34a853"/>
+        <a:srgbClr val="34A853"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="ff6d01"/>
+        <a:srgbClr val="FF6D01"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46bdc6"/>
+        <a:srgbClr val="46BDC6"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Sheets">
@@ -883,7 +904,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.62109375" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.08"/>
@@ -1237,7 +1258,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="7.68359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="7.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="5.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="10" width="8.94"/>
@@ -1489,7 +1510,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R1021"/>
-  <sheetFormatPr defaultColWidth="7.68359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="7.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="9.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="14.38"/>
@@ -4288,19 +4309,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultColWidth="12.8046875" defaultRowHeight="16.65" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="16.65" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="32" width="6.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="32" width="7.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="32" width="27.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="32" width="126.57"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="5" min="5" style="32" width="12.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="32" width="2.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="32" width="9.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="32" width="10.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="32" width="10.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="32" width="20.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="32" width="6.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="32" width="6.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="32" width="30.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="32" width="110.12"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="5" min="5" style="32" width="10.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="32" width="8.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="32" width="8.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="32" width="8.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="32" width="17.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4318,7 +4338,7 @@
       </c>
       <c r="E1" s="33"/>
       <c r="F1" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G1" s="33" t="n">
         <v>1</v>
@@ -4327,9 +4347,6 @@
         <v>1</v>
       </c>
       <c r="I1" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="J1" s="33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4347,190 +4364,270 @@
         <v>43</v>
       </c>
       <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34" t="s">
+      <c r="F2" s="34" t="s">
         <v>45</v>
       </c>
+      <c r="G2" s="35" t="s">
+        <v>82</v>
+      </c>
       <c r="H2" s="35" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I2" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="J2" s="35" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="36"/>
       <c r="B3" s="36" t="n">
-        <v>71001</v>
+        <v>0</v>
       </c>
       <c r="C3" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="36" t="s">
-        <v>86</v>
-      </c>
+      <c r="D3" s="36"/>
       <c r="E3" s="36"/>
-      <c r="F3" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36" t="n">
+        <v>71001</v>
+      </c>
       <c r="H3" s="36" t="n">
-        <v>71002</v>
+        <v>72003</v>
       </c>
       <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
     </row>
     <row r="4" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="36"/>
       <c r="B4" s="36" t="n">
+        <v>71001</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36" t="n">
         <v>71002</v>
       </c>
-      <c r="C4" s="36" t="s">
-        <v>88</v>
-      </c>
-      <c r="D4" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36" t="n">
-        <v>71003</v>
-      </c>
-      <c r="I4" s="36" t="n">
-        <v>72002</v>
-      </c>
-      <c r="J4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
     </row>
     <row r="5" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="36"/>
       <c r="B5" s="36" t="n">
+        <v>71002</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36" t="n">
         <v>71003</v>
       </c>
-      <c r="C5" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="D5" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="36"/>
       <c r="H5" s="36" t="n">
-        <v>71004</v>
+        <v>72002</v>
       </c>
       <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
     </row>
     <row r="6" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="36"/>
       <c r="B6" s="36" t="n">
+        <v>71003</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="36" t="n">
         <v>71004</v>
       </c>
-      <c r="C6" s="36" t="s">
-        <v>92</v>
-      </c>
-      <c r="D6" s="36" t="s">
-        <v>93</v>
-      </c>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" s="36"/>
       <c r="H6" s="36"/>
       <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
     </row>
     <row r="7" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="36"/>
       <c r="B7" s="36" t="n">
-        <v>72001</v>
+        <v>71004</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E7" s="36"/>
-      <c r="F7" s="36" t="s">
-        <v>87</v>
-      </c>
+      <c r="F7" s="36"/>
       <c r="G7" s="36"/>
       <c r="H7" s="36"/>
       <c r="I7" s="36"/>
-      <c r="J7" s="36" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="8" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="36"/>
       <c r="B8" s="36" t="n">
-        <v>72002</v>
+        <v>72001</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E8" s="36"/>
-      <c r="F8" s="36" t="s">
-        <v>87</v>
-      </c>
+      <c r="F8" s="36"/>
       <c r="G8" s="36"/>
       <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36" t="n">
+      <c r="I8" s="36" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="36"/>
       <c r="B9" s="36" t="n">
-        <v>72003</v>
+        <v>72002</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E9" s="36"/>
       <c r="F9" s="36"/>
       <c r="G9" s="36"/>
       <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I9" s="36" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="18.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="36"/>
       <c r="B10" s="36" t="n">
-        <v>73001</v>
+        <v>72003</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E10" s="36"/>
       <c r="F10" s="36"/>
       <c r="G10" s="36"/>
       <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36" t="n">
-        <v>3</v>
+      <c r="I10" s="36" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="36"/>
+      <c r="B11" s="36" t="n">
+        <v>73001</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>100</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="12" s="4" customFormat="true" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="36"/>
+      <c r="B12" s="36" t="n">
+        <v>72011</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" s="36" t="s">
+        <v>103</v>
+      </c>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36" t="n">
+        <v>72012</v>
+      </c>
+      <c r="I12" s="36" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="36"/>
+      <c r="B13" s="36" t="n">
+        <v>72012</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="36"/>
+      <c r="B14" s="36" t="n">
+        <v>72004</v>
+      </c>
+      <c r="C14" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="36"/>
+      <c r="B15" s="36" t="n">
+        <v>71011</v>
+      </c>
+      <c r="C15" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="36" t="n">
+        <v>1.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>